<commit_message>
Add researcher links, partners carousel; fix rotator descenders
Import website/LinkedIn links for PIs and staff from the researchers
spreadsheet, replace the partners grid with a full-bleed logo carousel,
and give the rotating word room for descenders.
</commit_message>
<xml_diff>
--- a/data/pi-links.template.xlsx
+++ b/data/pi-links.template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,6 +432,11 @@
           <t>LinkedIn</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,8 +444,6 @@
           <t>Prof. Gidi Grader</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -448,8 +451,6 @@
           <t>Prof. Oz Gazit</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
-      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -457,8 +458,6 @@
           <t>Prof. Moris Eisen</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -466,8 +465,6 @@
           <t>Prof. Michael Patrascu</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -475,8 +472,6 @@
           <t>Prof. David Eisenberg</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -484,17 +479,13 @@
           <t>Prof. Sabrina Spatari</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Prof. Maytal Caspari Toroker</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
+          <t>Prof. Maytal Caspary Toroker</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -502,8 +493,6 @@
           <t>Prof. Alon Grinberg Dana</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -511,8 +500,6 @@
           <t>Prof. Beni Cukurel</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -520,8 +507,6 @@
           <t>Prof. Joseph Lefkowitz</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -529,8 +514,34 @@
           <t>Prof. Dan Michaels</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Keren-Or Rosner</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Melad Atrash</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Victor Halperin</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Jawan Muhamed</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>